<commit_message>
Fix spreadsheet date imports, add printable PDF and consent-based resource measurement
</commit_message>
<xml_diff>
--- a/assets/downloads/13-week-cash-flow-forecast-template.xlsx
+++ b/assets/downloads/13-week-cash-flow-forecast-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="1" r:id="R95347431f26944b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="2" r:id="Ra573765cfca24e5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="1" r:id="R11f0c226aba84bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="2" r:id="R28a1135d97124034"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -339,8 +339,8 @@
       <x:c r="A3" s="1" t="str">
         <x:v>First Monday</x:v>
       </x:c>
-      <x:c r="B3" s="8" t="d">
-        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      <x:c r="B3" s="8" t="n">
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>
@@ -913,8 +913,8 @@
       <x:c r="A3" s="1" t="str">
         <x:v>First Monday</x:v>
       </x:c>
-      <x:c r="B3" s="8" t="d">
-        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      <x:c r="B3" s="8" t="n">
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>

</xml_diff>

<commit_message>
Fix template date imports and add PDF/download measurement (#175)
* Fix spreadsheet date imports, add printable PDF and consent-based resource measurement

* Exclude planner category links from product-click measurements
</commit_message>
<xml_diff>
--- a/assets/downloads/13-week-cash-flow-forecast-template.xlsx
+++ b/assets/downloads/13-week-cash-flow-forecast-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="1" r:id="R95347431f26944b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="2" r:id="Ra573765cfca24e5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="1" r:id="R11f0c226aba84bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="2" r:id="R28a1135d97124034"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -339,8 +339,8 @@
       <x:c r="A3" s="1" t="str">
         <x:v>First Monday</x:v>
       </x:c>
-      <x:c r="B3" s="8" t="d">
-        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      <x:c r="B3" s="8" t="n">
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>
@@ -913,8 +913,8 @@
       <x:c r="A3" s="1" t="str">
         <x:v>First Monday</x:v>
       </x:c>
-      <x:c r="B3" s="8" t="d">
-        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      <x:c r="B3" s="8" t="n">
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>

</xml_diff>